<commit_message>
feat(fmp): repoint REQ-23-D01 pipeline to RAW mcp.ledsone DB (order_management + inventory)
Sources all numbers + stock + Product ID from the raw ledsone schema via psycopg2
(fmp_fetch_raw.py, LED creds reach 169.58.91.229 = mcp.ledsone) - reconciled to the
cent against the warehouse. Grain aligned to (Product ID, SKU) per channel. Product
Name & Category carried as curated catalog labels by SKU. Adds fmp_query_raw.sql;
automation-ready. Rebuilt Excel + dashboard.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/development/abiraj_mini_aios_workbench/projects/PRJ-2026-020_fast-moving-products/evidence/final_outputs/REQ-23_fast-moving-products/REQ-23-D01_fast_moving_products.xlsx
+++ b/development/abiraj_mini_aios_workbench/projects/PRJ-2026-020_fast-moving-products/evidence/final_outputs/REQ-23_fast-moving-products/REQ-23-D01_fast_moving_products.xlsx
@@ -571,7 +571,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="56" customHeight="1">
+    <row r="4" ht="70" customHeight="1">
       <c r="A4" s="1" t="inlineStr">
         <is>
           <t>Data sources</t>
@@ -579,7 +579,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Sales/units/orders: public.order_transaction (source_name, market_place='Germany'). Product Name: inv_products.title / listing_data.title by SKU. Category: latest non-null order_transaction.category_name per SKU (~74% coverage; rest 'Uncategorised'). Current Stock: location_wise_inv_stock, location='Germany'.</t>
+          <t>RAW mcp.ledsone DB (read-only). Sales/units/orders: order_management.orders + order_item_info, joined to sub_source/source for channel (Amazon=1/eBay=2/Shopify=3), market_place='10' (Germany), status='Completed'. Current Stock: inventory.products + inventory.local_inventory_current_stock_location_wise, warehouse_location='Germany'. Product Name &amp; Category are curated catalog labels carried by SKU (raw combo titles are placeholders; category has no per-SKU raw home).</t>
         </is>
       </c>
     </row>
@@ -2152,7 +2152,7 @@
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>4 - 7W</t>
+          <t>4-7W Constant Current LED Driver, 300mA IP20 Rated Constant Current LED Driver Transformer, Converts AC85-265V into DC12-26V, IP20 Constant Current DC Transformers</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
@@ -2343,7 +2343,7 @@
         <v>73</v>
       </c>
       <c r="H4" s="9" t="n">
-        <v>629.03</v>
+        <v>629.04</v>
       </c>
       <c r="I4" s="8" t="n">
         <v>22</v>
@@ -2455,7 +2455,7 @@
         <v>62</v>
       </c>
       <c r="H6" s="9" t="n">
-        <v>467.78</v>
+        <v>467.79</v>
       </c>
       <c r="I6" s="8" t="n">
         <v>15</v>
@@ -2567,7 +2567,7 @@
         <v>54</v>
       </c>
       <c r="H8" s="9" t="n">
-        <v>378.38</v>
+        <v>378.39</v>
       </c>
       <c r="I8" s="8" t="n">
         <v>12</v>
@@ -2623,7 +2623,7 @@
         <v>18</v>
       </c>
       <c r="H9" s="13" t="n">
-        <v>183.18</v>
+        <v>183.19</v>
       </c>
       <c r="I9" s="12" t="n">
         <v>11</v>
@@ -3071,7 +3071,7 @@
         <v>10</v>
       </c>
       <c r="H17" s="13" t="n">
-        <v>181.33</v>
+        <v>181.34</v>
       </c>
       <c r="I17" s="12" t="n">
         <v>5</v>
@@ -3127,7 +3127,7 @@
         <v>11</v>
       </c>
       <c r="H18" s="9" t="n">
-        <v>175.31</v>
+        <v>175.3</v>
       </c>
       <c r="I18" s="8" t="n">
         <v>6</v>
@@ -3183,7 +3183,7 @@
         <v>10</v>
       </c>
       <c r="H19" s="13" t="n">
-        <v>148.95</v>
+        <v>148.92</v>
       </c>
       <c r="I19" s="12" t="n">
         <v>1</v>
@@ -3295,7 +3295,7 @@
         <v>11</v>
       </c>
       <c r="H21" s="13" t="n">
-        <v>49.48</v>
+        <v>49.49</v>
       </c>
       <c r="I21" s="12" t="n">
         <v>3</v>
@@ -3519,7 +3519,7 @@
         <v>8</v>
       </c>
       <c r="H25" s="17" t="n">
-        <v>116.88</v>
+        <v>116.91</v>
       </c>
       <c r="I25" s="16" t="n">
         <v>1</v>
@@ -3575,7 +3575,7 @@
         <v>11</v>
       </c>
       <c r="H26" s="9" t="n">
-        <v>92.06</v>
+        <v>92.03</v>
       </c>
       <c r="I26" s="8" t="n">
         <v>4</v>
@@ -3631,7 +3631,7 @@
         <v>17</v>
       </c>
       <c r="H27" s="13" t="n">
-        <v>172.31</v>
+        <v>172.29</v>
       </c>
       <c r="I27" s="12" t="n">
         <v>5</v>
@@ -4744,7 +4744,7 @@
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>4 - 7W</t>
+          <t>4-7W Constant Current LED Driver, 300mA IP20 Rated Constant Current LED Driver Transformer, Converts AC85-265V into DC12-26V, IP20 Constant Current DC Transformers</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
@@ -5418,7 +5418,7 @@
         <v>56</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>729.6799999999999</v>
+        <v>729.67</v>
       </c>
       <c r="J5" s="12" t="n">
         <v>987</v>
@@ -5443,7 +5443,7 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>IP67 15W Waterproof DC 12V LED Power Supply Driver Transformer AC 90-250V Flicker-free output, Outdoor transformer for garden lighting, pond water pumps</t>
+          <t>15W</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
@@ -5489,7 +5489,7 @@
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>LED Driver Power Supply 85V–265V DC Constant Current Transformer Adapter Flicker-Free Output For LED Strip Lights, LED Modules, and Power Accessories Indoor</t>
+          <t>12W</t>
         </is>
       </c>
       <c r="D7" s="11" t="inlineStr">
@@ -5535,7 +5535,7 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>E27 ST64 Vintage LED Dimmable  Bulbs, 4W Edison Light Bulb, 2700K Warm White, Amber Retro Style Energy Saving Filament Decorative Bulbs</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
@@ -5581,7 +5581,7 @@
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>LED Driver Power Supply 85V–265V DC Constant Current Transformer Adapter Flicker-Free Output For LED Strip Lights, LED Modules, and Power Accessories Indoor</t>
+          <t>4-7W Constant Current LED Driver, 300mA IP20 Rated Constant Current LED Driver Transformer, Converts AC85-265V into DC12-26V, IP20 Constant Current DC Transformers</t>
         </is>
       </c>
       <c r="D9" s="11" t="inlineStr">
@@ -5602,7 +5602,7 @@
         <v>38</v>
       </c>
       <c r="I9" s="13" t="n">
-        <v>226.87</v>
+        <v>226.88</v>
       </c>
       <c r="J9" s="12" t="n">
         <v>260</v>
@@ -5627,7 +5627,7 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Combo Default Title.</t>
+          <t>LEDSone Industrial Pendant Light Retro Chandelier Ceiling Light Vintage Lamp Ceiling Lighting Metal Shade for Restaurant Living Room Bedroom Kitchen Hallway Bar (Nero interno bianco)</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
@@ -5648,7 +5648,7 @@
         <v>31</v>
       </c>
       <c r="I10" s="9" t="n">
-        <v>629.03</v>
+        <v>629.04</v>
       </c>
       <c r="J10" s="8" t="n">
         <v>491</v>
@@ -5673,7 +5673,7 @@
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>E27 ST64 Vintage LED Dimmable  Bulbs, 8W Edison Light Bulb, 2700K Warm White, Amber Retro Style Energy Saving Filament Decorative Bulbs</t>
+          <t>1 PACK</t>
         </is>
       </c>
       <c r="D11" s="11" t="inlineStr">
@@ -5719,7 +5719,7 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>IP67 30W Waterproof DC 12V LED Power Supply Driver Transformer AC 90-250V Flicker-free output, Outdoor transformer for garden lighting, pond water pumps</t>
+          <t>30W</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
@@ -5765,7 +5765,7 @@
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>Black Colour Vintage Ceiling Rose Perfect for fabric flex cable, 100mm Metal Ceiling Light Fitting Plate with Accessories for Ceiling and Wall Lamp.</t>
+          <t>3.9 Inch Black Ceiling Canopy Kit Ceiling Plate, Modern Steel Canopy Kit Light Fixture for endant Light and Chandelier with All Hardware Includes Loop, Cross Bar and Mounting Screws.</t>
         </is>
       </c>
       <c r="D13" s="11" t="inlineStr">
@@ -5857,7 +5857,7 @@
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>DC 5V 50W 10Amp Power Supply Universal Regulated Switching AC to DC Converter AC110V/220V constant voltage Transformer Driver Adaptor for LED Strip Light, CCTV Camera Security System, Radio, Computer Project</t>
+          <t>50W</t>
         </is>
       </c>
       <c r="D15" s="11" t="inlineStr">
@@ -5903,7 +5903,7 @@
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>T connector</t>
+          <t>Boîte de jonction étanche IP68 - Connecteur de câble 3 voies - Connecteurs métalliques externes - Rallonge de boîte de jonction électrique - 3 voies pour câbles (1 paquet)</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
@@ -5949,7 +5949,7 @@
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>LEDSone Metalen Easy Fit Lampenkap Retro Industriële Plafond Verlichting Schaduw Opknoping Hanger Schaduw Lichtpunt voor Keuken Eetkamer Lichten E27 (Blauw)</t>
+          <t>LEDSone Metall Lampenschirm Retro Industrielle Deckenbeleuchtung Pendelleuchte (Schwarz Innen Weiß, 2 Packung)</t>
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr">
@@ -6087,7 +6087,7 @@
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>Light Socket E27 Bulb Socket Ceramics Lamp Holder Lampshades addable ES Screw Bulb Lamp holder</t>
+          <t>Black</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
@@ -6133,7 +6133,7 @@
       </c>
       <c r="C21" s="11" t="inlineStr">
         <is>
-          <t>DC VOLTAGE New Vintage Pendant Ceiling Shade Industrial Chandelier Flush Mount Lighting UK</t>
+          <t>Lampada a sospensione retrò E27 32 cm, lampada da soffitto in metallo, stile vintage, cavo regolabile - Faretto bianco per cucina, sala da pranzo, bar, caffetteria, ufficio (Verde)</t>
         </is>
       </c>
       <c r="D21" s="11" t="inlineStr">
@@ -6154,7 +6154,7 @@
         <v>22</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>467.78</v>
+        <v>467.79</v>
       </c>
       <c r="J21" s="12" t="n">
         <v>200</v>
@@ -6179,7 +6179,7 @@
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>IP67 150W Waterproof DC 12V LED Power Supply Driver Transformer AC 90-250V Flicker-free 2 output, Outdoor transformer for garden lighting, pond water pumps</t>
+          <t>12V 150W IP67 Waterproof LED Driver Transformer For Outdoor Lighting</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
@@ -6271,7 +6271,7 @@
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>Default Title</t>
+          <t>LEDSone Industrial Pendant Light Retro Chandelier Ceiling Light Vintage Lamp Ceiling Lighting Metal Shade for Restaurant Living Room Bedroom Kitchen Hallway Bar (Grigio)</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
@@ -6317,7 +6317,7 @@
       </c>
       <c r="C25" s="11" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Lámpara colgante industrial retro, lámpara de techo, lámpara vintage, iluminación de techo, pantalla de metal para (Negro, Sin bombilla)</t>
         </is>
       </c>
       <c r="D25" s="11" t="inlineStr">
@@ -6338,7 +6338,7 @@
         <v>22</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>427.43</v>
+        <v>427.44</v>
       </c>
       <c r="J25" s="12" t="n">
         <v>372</v>
@@ -6363,7 +6363,7 @@
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>IP67 36W Waterproof DC 12V LED Power Supply Driver Transformer AC 90-250V Flicker-free output, Outdoor transformer for garden lighting, pond water pumps</t>
+          <t>36W</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="C27" s="11" t="inlineStr">
         <is>
-          <t>Yellow Brass Light Chain Pendant Light Fixture Chain, Vintage 32mm x 17mm Lighting Hanging Chain for lighting Ceiling lights, Pendant lights, Lamp fixtures, Chandeliers, for light weight.</t>
+          <t>LEDSone Heavy Chandelier Copper Light Chain 32mm x 17mm for Lighting Ceiling Lights Pendant Hanging Chain (Yellow Brass)</t>
         </is>
       </c>
       <c r="D27" s="11" t="inlineStr">
@@ -6455,7 +6455,7 @@
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>Black / No</t>
+          <t>LEDSone Lámpara colgante de techo estilo retro industrial vintage con pantallas de cúpula curvada en color naranja, soporte E27 (Negro)</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
@@ -6476,7 +6476,7 @@
         <v>20</v>
       </c>
       <c r="I28" s="9" t="n">
-        <v>394</v>
+        <v>394.01</v>
       </c>
       <c r="J28" s="8" t="n">
         <v>372</v>

</xml_diff>